<commit_message>
[UPD] Updated corrected database
</commit_message>
<xml_diff>
--- a/data/daily_manual_rain_gage_data.xlsx
+++ b/data/daily_manual_rain_gage_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eiven\O2 Cloud\git\app-secar_meteo_data\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF109269-3C21-4191-A8C3-21D4E7882BFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1852AF9E-DCE8-46C8-9E0A-BB588B95B95E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Manual rain gage data" sheetId="1" r:id="rId1"/>
@@ -531,12 +531,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E4611"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14.5"/>
+  <dimension ref="A1:E4641"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="9.1796875" customWidth="1"/>
+    <col min="3" max="3" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -52512,6 +52512,339 @@
         <v>46249</v>
       </c>
       <c r="C4611">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4612" spans="1:3">
+      <c r="A4612" s="7">
+        <v>4610</v>
+      </c>
+      <c r="B4612" s="10">
+        <v>46250</v>
+      </c>
+      <c r="C4612">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4613" spans="1:3">
+      <c r="A4613" s="7">
+        <v>4611</v>
+      </c>
+      <c r="B4613" s="10">
+        <v>46251</v>
+      </c>
+      <c r="C4613">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4614" spans="1:3">
+      <c r="A4614" s="7">
+        <v>4612</v>
+      </c>
+      <c r="B4614" s="10">
+        <v>46252</v>
+      </c>
+      <c r="C4614">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4615" spans="1:3">
+      <c r="A4615" s="7">
+        <v>4613</v>
+      </c>
+      <c r="B4615" s="10">
+        <v>46253</v>
+      </c>
+      <c r="C4615">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4616" spans="1:3">
+      <c r="A4616" s="7">
+        <v>4614</v>
+      </c>
+      <c r="B4616" s="10">
+        <v>46254</v>
+      </c>
+      <c r="C4616">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4617" spans="1:3">
+      <c r="A4617" s="7">
+        <v>4615</v>
+      </c>
+      <c r="B4617" s="10">
+        <v>46255</v>
+      </c>
+      <c r="C4617">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4618" spans="1:3">
+      <c r="A4618" s="7">
+        <v>4616</v>
+      </c>
+      <c r="B4618" s="10">
+        <v>46256</v>
+      </c>
+      <c r="C4618">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4619" spans="1:3">
+      <c r="A4619" s="7">
+        <v>4617</v>
+      </c>
+      <c r="B4619" s="10">
+        <v>46257</v>
+      </c>
+      <c r="C4619">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4620" spans="1:3">
+      <c r="A4620" s="7">
+        <v>4618</v>
+      </c>
+      <c r="B4620" s="10">
+        <v>46258</v>
+      </c>
+      <c r="C4620">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4621" spans="1:3">
+      <c r="A4621" s="7">
+        <v>4619</v>
+      </c>
+      <c r="B4621" s="10">
+        <v>46259</v>
+      </c>
+      <c r="C4621">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4622" spans="1:3">
+      <c r="A4622" s="7">
+        <v>4620</v>
+      </c>
+      <c r="B4622" s="10">
+        <v>46260</v>
+      </c>
+      <c r="C4622">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4623" spans="1:3">
+      <c r="A4623" s="7">
+        <v>4621</v>
+      </c>
+      <c r="B4623" s="10">
+        <v>46261</v>
+      </c>
+      <c r="C4623">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4624" spans="1:3">
+      <c r="A4624" s="7">
+        <v>4622</v>
+      </c>
+      <c r="B4624" s="10">
+        <v>46262</v>
+      </c>
+      <c r="C4624">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4625" spans="1:5">
+      <c r="A4625" s="7">
+        <v>4623</v>
+      </c>
+      <c r="B4625" s="10">
+        <v>46263</v>
+      </c>
+      <c r="C4625">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4626" spans="1:5">
+      <c r="A4626" s="7">
+        <v>4624</v>
+      </c>
+      <c r="B4626" s="10">
+        <v>46264</v>
+      </c>
+      <c r="C4626">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4627" spans="1:5">
+      <c r="A4627" s="7">
+        <v>4625</v>
+      </c>
+      <c r="B4627" s="10">
+        <v>46265</v>
+      </c>
+      <c r="C4627">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4628" spans="1:5">
+      <c r="A4628" s="7">
+        <v>4626</v>
+      </c>
+      <c r="B4628" s="10">
+        <v>46266</v>
+      </c>
+      <c r="C4628">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4629" spans="1:5">
+      <c r="A4629" s="7">
+        <v>4627</v>
+      </c>
+      <c r="B4629" s="10">
+        <v>46267</v>
+      </c>
+      <c r="C4629">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4630" spans="1:5">
+      <c r="A4630" s="7">
+        <v>4628</v>
+      </c>
+      <c r="B4630" s="10">
+        <v>46268</v>
+      </c>
+      <c r="C4630">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4631" spans="1:5">
+      <c r="A4631" s="7">
+        <v>4629</v>
+      </c>
+      <c r="B4631" s="10">
+        <v>46269</v>
+      </c>
+      <c r="C4631">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4632" spans="1:5">
+      <c r="A4632" s="7">
+        <v>4630</v>
+      </c>
+      <c r="B4632" s="10">
+        <v>46270</v>
+      </c>
+      <c r="C4632">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4633" spans="1:5">
+      <c r="A4633" s="7">
+        <v>4631</v>
+      </c>
+      <c r="B4633" s="10">
+        <v>46271</v>
+      </c>
+      <c r="C4633">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4634" spans="1:5">
+      <c r="A4634" s="7">
+        <v>4632</v>
+      </c>
+      <c r="B4634" s="10">
+        <v>46272</v>
+      </c>
+      <c r="C4634">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4635" spans="1:5">
+      <c r="A4635" s="7">
+        <v>4633</v>
+      </c>
+      <c r="B4635" s="10">
+        <v>46273</v>
+      </c>
+      <c r="C4635">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4636" spans="1:5">
+      <c r="A4636" s="7">
+        <v>4634</v>
+      </c>
+      <c r="B4636" s="10">
+        <v>46274</v>
+      </c>
+      <c r="C4636">
+        <v>14.2</v>
+      </c>
+      <c r="E4636">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4637" spans="1:5">
+      <c r="A4637" s="7">
+        <v>4635</v>
+      </c>
+      <c r="B4637" s="10">
+        <v>46275</v>
+      </c>
+      <c r="C4637">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4638" spans="1:5">
+      <c r="A4638" s="7">
+        <v>4636</v>
+      </c>
+      <c r="B4638" s="10">
+        <v>46276</v>
+      </c>
+      <c r="C4638">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4639" spans="1:5">
+      <c r="A4639" s="7">
+        <v>4637</v>
+      </c>
+      <c r="B4639" s="10">
+        <v>46277</v>
+      </c>
+      <c r="C4639">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4640" spans="1:5">
+      <c r="A4640" s="7">
+        <v>4638</v>
+      </c>
+      <c r="B4640" s="10">
+        <v>46278</v>
+      </c>
+      <c r="C4640">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4641" spans="1:3">
+      <c r="A4641" s="7">
+        <v>4639</v>
+      </c>
+      <c r="B4641" s="10">
+        <v>46279</v>
+      </c>
+      <c r="C4641">
         <v>0</v>
       </c>
     </row>
@@ -52523,14 +52856,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E31"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="43" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="42.95" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="11.453125" customWidth="1"/>
-    <col min="2" max="2" width="13.54296875" customWidth="1"/>
-    <col min="3" max="3" width="17.1796875" customWidth="1"/>
-    <col min="4" max="4" width="18.81640625" customWidth="1"/>
-    <col min="5" max="5" width="37.1796875" customWidth="1"/>
-    <col min="6" max="6" width="34.54296875" customWidth="1"/>
+    <col min="1" max="1" width="11.42578125" customWidth="1"/>
+    <col min="2" max="2" width="13.5703125" customWidth="1"/>
+    <col min="3" max="3" width="17.140625" customWidth="1"/>
+    <col min="4" max="4" width="18.85546875" customWidth="1"/>
+    <col min="5" max="5" width="37.140625" customWidth="1"/>
+    <col min="6" max="6" width="34.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="21" customHeight="1">
@@ -52567,7 +52900,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="43" customHeight="1">
+    <row r="3" spans="1:5" ht="42.95" customHeight="1">
       <c r="A3" s="2">
         <v>41753</v>
       </c>
@@ -52584,7 +52917,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="43" customHeight="1">
+    <row r="4" spans="1:5" ht="42.95" customHeight="1">
       <c r="A4" s="2">
         <v>42001</v>
       </c>
@@ -52601,7 +52934,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="43" customHeight="1">
+    <row r="5" spans="1:5" ht="42.95" customHeight="1">
       <c r="A5" s="2">
         <v>42002</v>
       </c>
@@ -52618,7 +52951,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="43" customHeight="1">
+    <row r="6" spans="1:5" ht="42.95" customHeight="1">
       <c r="A6" s="2">
         <v>41643</v>
       </c>
@@ -52635,7 +52968,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="43" customHeight="1">
+    <row r="7" spans="1:5" ht="42.95" customHeight="1">
       <c r="A7" s="2">
         <v>41668</v>
       </c>
@@ -52652,7 +52985,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="43" customHeight="1">
+    <row r="8" spans="1:5" ht="42.95" customHeight="1">
       <c r="A8" s="2">
         <v>41675</v>
       </c>
@@ -52666,7 +52999,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="43" customHeight="1">
+    <row r="9" spans="1:5" ht="42.95" customHeight="1">
       <c r="A9" s="2">
         <v>42234</v>
       </c>
@@ -52680,7 +53013,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="43" customHeight="1">
+    <row r="10" spans="1:5" ht="42.95" customHeight="1">
       <c r="A10" s="2">
         <v>42372</v>
       </c>
@@ -52694,7 +53027,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="43" customHeight="1">
+    <row r="11" spans="1:5" ht="42.95" customHeight="1">
       <c r="A11" s="2">
         <v>42407</v>
       </c>
@@ -52708,7 +53041,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="43" customHeight="1">
+    <row r="12" spans="1:5" ht="42.95" customHeight="1">
       <c r="A12" s="2">
         <v>42415</v>
       </c>
@@ -52722,7 +53055,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="43" customHeight="1">
+    <row r="13" spans="1:5" ht="42.95" customHeight="1">
       <c r="A13" s="2">
         <v>42427</v>
       </c>
@@ -52736,7 +53069,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="43" customHeight="1">
+    <row r="14" spans="1:5" ht="42.95" customHeight="1">
       <c r="A14" s="2">
         <v>42439</v>
       </c>
@@ -52750,7 +53083,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="43" customHeight="1">
+    <row r="15" spans="1:5" ht="42.95" customHeight="1">
       <c r="A15" s="2">
         <v>42444</v>
       </c>
@@ -52764,7 +53097,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="43" customHeight="1">
+    <row r="16" spans="1:5" ht="42.95" customHeight="1">
       <c r="A16" s="2">
         <v>42448</v>
       </c>
@@ -52778,7 +53111,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="43" customHeight="1">
+    <row r="17" spans="1:4" ht="42.95" customHeight="1">
       <c r="A17" s="2">
         <v>42468</v>
       </c>
@@ -52792,7 +53125,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="43" customHeight="1">
+    <row r="18" spans="1:4" ht="42.95" customHeight="1">
       <c r="A18" s="2">
         <v>42480</v>
       </c>
@@ -52806,7 +53139,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="43" customHeight="1">
+    <row r="19" spans="1:4" ht="42.95" customHeight="1">
       <c r="A19" s="2">
         <v>42491</v>
       </c>
@@ -52820,7 +53153,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="43" customHeight="1">
+    <row r="20" spans="1:4" ht="42.95" customHeight="1">
       <c r="A20" s="2">
         <v>42549</v>
       </c>
@@ -52834,7 +53167,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="43" customHeight="1">
+    <row r="21" spans="1:4" ht="42.95" customHeight="1">
       <c r="A21" s="2">
         <v>42550</v>
       </c>
@@ -52848,7 +53181,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="43" customHeight="1">
+    <row r="22" spans="1:4" ht="42.95" customHeight="1">
       <c r="A22" s="2">
         <v>43158</v>
       </c>
@@ -52862,7 +53195,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="43" customHeight="1">
+    <row r="23" spans="1:4" ht="42.95" customHeight="1">
       <c r="A23" s="2">
         <v>43159</v>
       </c>
@@ -52876,7 +53209,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="24" spans="1:4" ht="43" customHeight="1">
+    <row r="24" spans="1:4" ht="42.95" customHeight="1">
       <c r="A24" s="2">
         <v>43160</v>
       </c>
@@ -52890,7 +53223,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="43" customHeight="1">
+    <row r="25" spans="1:4" ht="42.95" customHeight="1">
       <c r="A25" s="2">
         <v>43161</v>
       </c>
@@ -52904,7 +53237,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="26" spans="1:4" ht="43" customHeight="1">
+    <row r="26" spans="1:4" ht="42.95" customHeight="1">
       <c r="A26" s="2">
         <v>43358</v>
       </c>
@@ -52918,7 +53251,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="43" customHeight="1">
+    <row r="27" spans="1:4" ht="42.95" customHeight="1">
       <c r="A27" s="2">
         <v>43360</v>
       </c>
@@ -52932,7 +53265,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="43" customHeight="1">
+    <row r="28" spans="1:4" ht="42.95" customHeight="1">
       <c r="A28" s="2">
         <v>43413</v>
       </c>
@@ -52946,7 +53279,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="43" customHeight="1">
+    <row r="29" spans="1:4" ht="42.95" customHeight="1">
       <c r="A29" s="2">
         <v>43418</v>
       </c>
@@ -52960,7 +53293,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="43" customHeight="1">
+    <row r="30" spans="1:4" ht="42.95" customHeight="1">
       <c r="A30" s="2">
         <v>43430</v>
       </c>
@@ -52974,7 +53307,7 @@
         <v>45949</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="43" customHeight="1">
+    <row r="31" spans="1:4" ht="42.95" customHeight="1">
       <c r="A31" s="2">
         <v>43654</v>
       </c>

</xml_diff>